<commit_message>
ajustes de la ia y de los backups del inventario
</commit_message>
<xml_diff>
--- a/Inventario_Quiosco.xlsx
+++ b/Inventario_Quiosco.xlsx
@@ -1,102 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD3505D56A61A2B93521510344D07F24C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CDB83FF-1A2D-4DCC-8235-7DA6A1EA6AEA}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>Código</t>
-  </si>
-  <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>Precio Venta</t>
-  </si>
-  <si>
-    <t>Stock Actual</t>
-  </si>
-  <si>
-    <t>Stock Mínimo</t>
-  </si>
-  <si>
-    <t>Fecha Vencimiento</t>
-  </si>
-  <si>
-    <t>alfajor rasta</t>
-  </si>
-  <si>
-    <t>2026-07-01</t>
-  </si>
-  <si>
-    <t>12426543.0</t>
-  </si>
-  <si>
-    <t>Lays originales</t>
-  </si>
-  <si>
-    <t>2026-06-26</t>
-  </si>
-  <si>
-    <t>cocacola de 500ml</t>
-  </si>
-  <si>
-    <t>2026-12-15</t>
-  </si>
-  <si>
-    <t>8723659</t>
-  </si>
-  <si>
-    <t>don satur saladas</t>
-  </si>
-  <si>
-    <t>2026-06-24</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -115,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -417,102 +408,188 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Precio Venta</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Stock Actual</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Stock Mínimo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fecha Vencimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>alfajor rasta</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>12426543.0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lays originales</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cocacola de 500ml</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="B2" t="s">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8723659.0</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>don satur saladas</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="n">
         <v>6</v>
       </c>
-      <c r="C2">
-        <v>1000</v>
-      </c>
-      <c r="D2">
-        <v>9</v>
-      </c>
-      <c r="E2">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>6834593.0</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>oreos</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3">
-        <v>3000</v>
-      </c>
-      <c r="D3">
-        <v>6</v>
-      </c>
-      <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>3500</v>
-      </c>
-      <c r="D4">
-        <v>40</v>
-      </c>
-      <c r="E4">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fantas de 500ml</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" t="n">
         <v>5</v>
       </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5">
-        <v>2000</v>
-      </c>
-      <c r="D5">
-        <v>7</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5" t="s">
-        <v>15</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustes de v1 beta
</commit_message>
<xml_diff>
--- a/Inventario_Quiosco.xlsx
+++ b/Inventario_Quiosco.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>24634645.0</t>
+          <t>7798397444202.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,7 +463,7 @@
         <v>1000</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
@@ -477,7 +477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12426543.0</t>
+          <t>7790310984031.0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,7 +529,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>8723659.0</t>
+          <t>7795735000328.0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -541,7 +541,7 @@
         <v>2000</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>6</v>
@@ -555,7 +555,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6834593.0</t>
+          <t>7622300864934.0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -567,7 +567,7 @@
         <v>2500</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
@@ -581,7 +581,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23526346.0</t>
+          <t>7790895000836</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,6 +603,54 @@
           <t>2026-09-23</t>
         </is>
       </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7790895650833.0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>coca 600ml</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7790580424565</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>gomitas mogul de ositos de 80g</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>